<commit_message>
Move Kotak BizLabs to Later: DPIIT won't be ready by 6 Oct
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KyDhbraNbwSeUjcrXQ23W5
</commit_message>
<xml_diff>
--- a/TF_PreSeed_Investor_List_30Sep2026.xlsx
+++ b/TF_PreSeed_Investor_List_30Sep2026.xlsx
@@ -709,14 +709,14 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SIDBI Innovation Challenge closes 16 Oct 2026. It fits if TF is pitched as AI-led market access for small restaurants (MSMEs). With Kotak BizLabs (6 Oct) and YC (2 Nov), it is one of three hard deadlines right now.</t>
+          <t>SIDBI Innovation Challenge closes 16 Oct 2026. It fits if TF is pitched as AI-led market access for small restaurants (MSMEs). With YC (2 Nov), it is one of two hard deadlines right now.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Kotak BizLabs Season 3 (grant up to Rs 30L, no equity) closes 6 Oct 2026 and needs DPIIT recognition by then. Only realistic if DPIIT lands this week, or if MSM Global already has it. Pick IIMCIP Kolkata as the partner and frame TF as fintech or inclusive tech.</t>
+          <t>Kotak BizLabs Season 3 (grant up to Rs 30L, no equity) closes 6 Oct 2026. TF will miss it because DPIIT recognition won't be ready. Watch for Season 4; it is a strong fit once DPIIT is in place.</t>
         </is>
       </c>
     </row>
@@ -14005,9 +14005,9 @@
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>A: apply first</t>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Later: next round</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -14082,7 +14082,11 @@
         </is>
       </c>
       <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>Missed Season 3 (no DPIIT by 6 Oct). Target Season 4 once Table Foundry Pvt Ltd has DPIIT recognition.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">

</xml_diff>